<commit_message>
fix useMemo errors, fix image routes, add harbinger setup for local hotseat, add random-spell to toolbox and dedicated endpoint to quickly call it up
</commit_message>
<xml_diff>
--- a/exports/gothic-set.xlsx
+++ b/exports/gothic-set.xlsx
@@ -483,7 +483,7 @@
         <v>Avatar</v>
       </c>
       <c r="C2" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D2" t="str">
         <v>None</v>
@@ -539,7 +539,7 @@
         <v>Avatar</v>
       </c>
       <c r="C3" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D3" t="str">
         <v>None</v>
@@ -595,7 +595,7 @@
         <v>Avatar</v>
       </c>
       <c r="C4" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D4" t="str">
         <v>None</v>
@@ -651,7 +651,7 @@
         <v>Avatar</v>
       </c>
       <c r="C5" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D5" t="str">
         <v>None</v>
@@ -707,7 +707,7 @@
         <v>Avatar</v>
       </c>
       <c r="C6" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D6" t="str">
         <v>None</v>
@@ -763,7 +763,7 @@
         <v>Avatar</v>
       </c>
       <c r="C7" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D7" t="str">
         <v>None</v>
@@ -819,7 +819,7 @@
         <v>Avatar</v>
       </c>
       <c r="C8" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D8" t="str">
         <v>None</v>
@@ -875,7 +875,7 @@
         <v>Avatar</v>
       </c>
       <c r="C9" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D9" t="str">
         <v>None</v>
@@ -931,7 +931,7 @@
         <v>Avatar</v>
       </c>
       <c r="C10" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D10" t="str">
         <v>None</v>
@@ -987,7 +987,7 @@
         <v>Avatar</v>
       </c>
       <c r="C11" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D11" t="str">
         <v>None</v>
@@ -1043,7 +1043,7 @@
         <v>Avatar</v>
       </c>
       <c r="C12" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D12" t="str">
         <v>None</v>
@@ -1099,7 +1099,7 @@
         <v>Avatar</v>
       </c>
       <c r="C13" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D13" t="str">
         <v>None</v>
@@ -1155,7 +1155,7 @@
         <v>Avatar</v>
       </c>
       <c r="C14" t="str">
-        <v/>
+        <v>Unique</v>
       </c>
       <c r="D14" t="str">
         <v>None</v>

</xml_diff>